<commit_message>
el matloub file updated
</commit_message>
<xml_diff>
--- a/el matloub machine learning.xlsx
+++ b/el matloub machine learning.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8280"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="el matloub machine learning" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>le projet dédié pour qui ?? médecin ,radiolyse …</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t xml:space="preserve"> the first dso is based on the one that came in the report , the others were brainstormed by the group </t>
+  </si>
+  <si>
+    <t xml:space="preserve">the project will contribute a lot to society and the medical and health domains </t>
   </si>
 </sst>
 </file>
@@ -1239,7 +1242,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -1342,6 +1345,11 @@
         <v>19</v>
       </c>
     </row>
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>